<commit_message>
Add software and speaking pages with dynamic content loading
- Created a new software page (software-page.qmd) that dynamically loads repositories from GitHub, displaying relevant information such as language, stars, and descriptions.
- Implemented a loading spinner and error handling for GitHub API requests.
- Added a new speaking page (speaking-page.qmd) that lists selected public speaking occasions, including talks and posters, with links to related materials.
- Integrated a timeline visualization for speaking events and a map to show conference locations.
- Included CSS for styling the software and speaking pages.
- Added a new image (uncertainty.png) to the projects directory.
</commit_message>
<xml_diff>
--- a/speaking/conferences.xlsx
+++ b/speaking/conferences.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kuleuven-my.sharepoint.com/personal/lasai_barrenadataleb_kuleuven_be/Documents/Documentos e informacion/Trabajo/Webpage_quarto/conferences/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kuleuven-my.sharepoint.com/personal/lasai_barrenadataleb_kuleuven_be/Documents/Documentos e informacion/Trabajo/Webpage_quarto - AI/speaking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="11_F25DC773A252ABDACC10489D719C6A665ADE58F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A16C359F-1C30-425E-B75F-D7E019502747}"/>
+  <xr:revisionPtr revIDLastSave="211" documentId="11_F25DC773A252ABDACC10489D719C6A665ADE58F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59231FE7-F0E5-460B-BAE9-DC590B31E41D}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="60">
   <si>
     <t>Location</t>
   </si>
@@ -78,9 +78,6 @@
     <t>Poster</t>
   </si>
   <si>
-    <t>Presentation</t>
-  </si>
-  <si>
     <t>Head-to-head comparisons of RMI and ADNEX model to diagnose ovarian malignancy: systematic review and meta-analysis</t>
   </si>
   <si>
@@ -117,15 +114,9 @@
     <t>Link_2_name</t>
   </si>
   <si>
-    <t>Abstract</t>
-  </si>
-  <si>
     <t>https://github.com/LasaiBarrenada/web_resources/blob/6620d40724dd436b0f2825cd91cad5181813a304/DRAWING%20MULTICENTER%20CALIBRATION%20CURVES%20w.pdf</t>
   </si>
   <si>
-    <t>https://obgyn.onlinelibrary.wiley.com/doi/10.1002/uog.26336</t>
-  </si>
-  <si>
     <t>https://github.com/LasaiBarrenada/web_resources/blob/6620d40724dd436b0f2825cd91cad5181813a304/202310%20ISUOG%20Seul.pptx</t>
   </si>
   <si>
@@ -136,16 +127,102 @@
   </si>
   <si>
     <t>Link_2</t>
+  </si>
+  <si>
+    <t>https://github.com/LasaiBarrenada/web_resources/blob/main/posterISCB2024_V2.pdf</t>
+  </si>
+  <si>
+    <t>New Orleans</t>
+  </si>
+  <si>
+    <t>ENAR</t>
+  </si>
+  <si>
+    <t>ENAR spring meeting</t>
+  </si>
+  <si>
+    <t>Oral presentation</t>
+  </si>
+  <si>
+    <t>The Fundamental Problem of Individual Risk Estimation for Health AI</t>
+  </si>
+  <si>
+    <t>Birmingham</t>
+  </si>
+  <si>
+    <t>Methods for Evaluating Models, Tests And Biomarkers</t>
+  </si>
+  <si>
+    <t>MEMTAB</t>
+  </si>
+  <si>
+    <t>Combining calibration plots from multiple centers or datasets</t>
+  </si>
+  <si>
+    <t>Paper</t>
+  </si>
+  <si>
+    <t>https://diagnprognres.biomedcentral.com/articles/10.1186/s41512-024-00177-1</t>
+  </si>
+  <si>
+    <t>https://bmjmedicine.bmj.com/content/3/1/e000817</t>
+  </si>
+  <si>
+    <t>Preprint</t>
+  </si>
+  <si>
+    <t>Slides</t>
+  </si>
+  <si>
+    <t>https://github.com/LasaiBarrenada/web_resources/blob/main/15.42%20-%20Mr%20Lasai%20Barre%C3%B1ada%20-%20%5BOP06.01%5D.pdf</t>
+  </si>
+  <si>
+    <t>https://github.com/LasaiBarrenada/web_resources/blob/main/ENAR_2025_forPDF.html</t>
+  </si>
+  <si>
+    <t>https://github.com/LasaiBarrenada/web_resources/blob/main/ClusteredCalibration%20MEMTAB%20V2%20Lasai.pdf</t>
+  </si>
+  <si>
+    <t>Cancun</t>
+  </si>
+  <si>
+    <t>ADNEX2: An updated ADNEX model</t>
+  </si>
+  <si>
+    <t>Slides (NA)</t>
+  </si>
+  <si>
+    <t>Preprint (NA)</t>
+  </si>
+  <si>
+    <t>Bilbao</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2506.17141</t>
+  </si>
+  <si>
+    <t>https://www.cambridge.org/core/journals/research-synthesis-methods/article/clustered-flexible-calibration-plots-for-binary-outcomes-using-random-effects-modeling/FE857DCCAD4A37B60EF819F26B2F9411</t>
+  </si>
+  <si>
+    <t>https://bmjopen.bmj.com/content/15/10/e104141</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -168,13 +245,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -188,10 +268,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -457,20 +533,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.44140625" customWidth="1"/>
-    <col min="8" max="8" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.42578125" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -488,30 +564,30 @@
         <v>15</v>
       </c>
       <c r="H1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" t="s">
         <v>28</v>
       </c>
-      <c r="I1" t="s">
-        <v>29</v>
-      </c>
       <c r="J1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="K1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E2">
         <v>2023</v>
@@ -523,24 +599,30 @@
         <v>16</v>
       </c>
       <c r="H2" t="s">
+        <v>44</v>
+      </c>
+      <c r="I2" t="s">
         <v>16</v>
       </c>
       <c r="J2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="K2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E3">
         <v>2023</v>
@@ -552,24 +634,30 @@
         <v>16</v>
       </c>
       <c r="H3" t="s">
+        <v>44</v>
+      </c>
+      <c r="I3" t="s">
         <v>16</v>
       </c>
       <c r="J3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="K3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E4">
         <v>2023</v>
@@ -578,33 +666,33 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="H4" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K4" t="s">
         <v>30</v>
       </c>
-      <c r="I4" t="s">
-        <v>17</v>
-      </c>
-      <c r="J4" t="s">
-        <v>32</v>
-      </c>
-      <c r="K4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E5">
         <v>2024</v>
@@ -613,27 +701,33 @@
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="H5" t="s">
-        <v>17</v>
+        <v>44</v>
+      </c>
+      <c r="I5" t="s">
+        <v>48</v>
       </c>
       <c r="J5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="K5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6">
         <v>2024</v>
@@ -645,21 +739,30 @@
         <v>16</v>
       </c>
       <c r="H6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J6" t="s">
+        <v>58</v>
+      </c>
+      <c r="K6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
         <v>8</v>
       </c>
       <c r="D7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E7">
         <v>2024</v>
@@ -668,13 +771,153 @@
         <v>9</v>
       </c>
       <c r="G7" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="H7" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="I7" t="s">
-        <v>17</v>
+        <v>48</v>
+      </c>
+      <c r="J7" t="s">
+        <v>59</v>
+      </c>
+      <c r="K7" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8">
+        <v>2025</v>
+      </c>
+      <c r="F8">
+        <v>3</v>
+      </c>
+      <c r="G8" t="s">
+        <v>38</v>
+      </c>
+      <c r="H8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I8" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" t="s">
+        <v>57</v>
+      </c>
+      <c r="K8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9">
+        <v>2025</v>
+      </c>
+      <c r="F9">
+        <v>4</v>
+      </c>
+      <c r="G9" t="s">
+        <v>38</v>
+      </c>
+      <c r="H9" t="s">
+        <v>44</v>
+      </c>
+      <c r="I9" t="s">
+        <v>48</v>
+      </c>
+      <c r="J9" t="s">
+        <v>58</v>
+      </c>
+      <c r="K9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10">
+        <v>2025</v>
+      </c>
+      <c r="F10">
+        <v>9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>38</v>
+      </c>
+      <c r="H10" t="s">
+        <v>55</v>
+      </c>
+      <c r="I10" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11">
+        <v>2026</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>38</v>
+      </c>
+      <c r="H11" t="s">
+        <v>47</v>
+      </c>
+      <c r="I11" t="s">
+        <v>48</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="K11" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -682,7 +925,10 @@
     <sortCondition ref="E2:E7"/>
     <sortCondition ref="F2:F7"/>
   </sortState>
+  <hyperlinks>
+    <hyperlink ref="J11" r:id="rId1" xr:uid="{0B3F84ED-8380-4963-8ECC-458C04B0DE86}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>